<commit_message>
minor test results added, code run for paper
</commit_message>
<xml_diff>
--- a/code/test results.xlsx
+++ b/code/test results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bradl\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bradl\Desktop\uni\final-project\code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0B596A1-5B2A-45E9-AAF4-F7378B2572D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D7E0847-178E-439C-955E-D41618E34718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{8A721CCB-E596-4063-BEBF-8402B06F69EA}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1315" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1314" uniqueCount="151">
   <si>
     <t>test number</t>
   </si>
@@ -542,9 +542,6 @@
   </si>
   <si>
     <t>above 2 tests but on SCIAMA</t>
-  </si>
-  <si>
-    <t>62 .18%</t>
   </si>
   <si>
     <t>scaled mel spectrogram values to be
@@ -643,7 +640,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -690,77 +687,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="42">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF630D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF630D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF630D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="33">
     <dxf>
       <fill>
         <patternFill>
@@ -1060,40 +991,40 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BDC20197-0D11-4F96-98C6-561676E67A6E}" name="Table1" displayName="Table1" ref="A2:AB142" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BDC20197-0D11-4F96-98C6-561676E67A6E}" name="Table1" displayName="Table1" ref="A2:AB142" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
   <autoFilter ref="A2:AB142" xr:uid="{BDC20197-0D11-4F96-98C6-561676E67A6E}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A35:AB76">
     <sortCondition ref="C2:C80"/>
   </sortState>
   <tableColumns count="28">
-    <tableColumn id="1" xr3:uid="{3318AD16-53B6-4688-8184-DCAE4D7989CC}" name="test number" dataDxfId="39"/>
-    <tableColumn id="26" xr3:uid="{36FCCC2D-6AA9-4D59-9607-CFE4E77F428F}" name="model iteration" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{6162A6E9-56C2-4DFE-8497-138E33277B23}" name="folders" dataDxfId="37"/>
-    <tableColumn id="24" xr3:uid="{84500DC1-61E5-441B-9BB7-98403DAEDDA3}" name="single or multi label" dataDxfId="36"/>
-    <tableColumn id="23" xr3:uid="{D53465F0-58BB-492A-A264-D9F6F9AD3C77}" name="file rating threshold" dataDxfId="35"/>
-    <tableColumn id="28" xr3:uid="{8B631FC7-380A-498A-87D1-A5A5CDE1B184}" name="sampling rate (hz)" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{455DD90A-7B3B-4AE3-B08F-EF626809FA12}" name="sound length (secs)" dataDxfId="33"/>
-    <tableColumn id="16" xr3:uid="{BE562B7A-09E8-48B6-87F1-F9358A9B6D5B}" name="files per folder threshold" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{E3C34C6B-84EB-4093-B2F3-6A3FEA8E014C}" name="sound clips per file threshold" dataDxfId="31"/>
-    <tableColumn id="27" xr3:uid="{191D39FF-C4F8-4DBA-B0D0-9163B957A029}" name="variance threshold" dataDxfId="30"/>
-    <tableColumn id="25" xr3:uid="{E5B8107D-0DF4-4EA1-ADD9-375779D45EF4}" name="mean db threshold" dataDxfId="29"/>
-    <tableColumn id="19" xr3:uid="{864FBBD1-F7F9-4946-B210-D69AFB5835DC}" name="test size" dataDxfId="28"/>
-    <tableColumn id="22" xr3:uid="{2B2C8707-3EBF-4F34-8873-79CDF32B12F6}" name="sampling" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{F22E151A-20C9-4BD4-9330-289A7FFEA185}" name="sound clips" dataDxfId="26"/>
-    <tableColumn id="18" xr3:uid="{5798ECBB-EF37-49E5-8484-9B35165F789E}" name="epochs" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{FCBAD803-5AC6-4170-96E5-CDADD42AAFE6}" name="loss function" dataDxfId="24"/>
-    <tableColumn id="7" xr3:uid="{28105F38-9933-41DD-903D-59C6CB55BAC1}" name="optimizer" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{EB347492-3ECD-4D09-9D3B-70F1B3841DE0}" name="learning rate" dataDxfId="22"/>
-    <tableColumn id="9" xr3:uid="{E8435981-3E1D-4BD4-B5A5-B92A95E47B32}" name="momentum" dataDxfId="21"/>
-    <tableColumn id="10" xr3:uid="{6CFBA716-45FB-401C-A304-C38379448F6E}" name="dropout rate" dataDxfId="20"/>
-    <tableColumn id="11" xr3:uid="{696423D6-C6E9-46A6-845B-0AF07B48592B}" name="batch size" dataDxfId="19"/>
-    <tableColumn id="12" xr3:uid="{7FD1D4E4-3292-4AA1-9BCC-2B94A81E0391}" name="training accuracy %" dataDxfId="18"/>
-    <tableColumn id="13" xr3:uid="{8EE7A374-9D10-4C25-9169-E97C46453BAF}" name="testing accuracy %" dataDxfId="17"/>
-    <tableColumn id="14" xr3:uid="{E1A45F5D-7C07-400E-8A62-BFF33A480A4C}" name="gpu train time (secs)" dataDxfId="16"/>
-    <tableColumn id="20" xr3:uid="{B80BC466-5D5A-48F1-9455-63991D7EF174}" name="top-5 accuracy" dataDxfId="15"/>
-    <tableColumn id="21" xr3:uid="{E7EF58AA-8977-49AA-AE41-D484359C41A5}" name="tested on?" dataDxfId="14"/>
-    <tableColumn id="15" xr3:uid="{26BF47AC-1BE1-47B7-86FA-94CD5B2EA529}" name="other changes" dataDxfId="13"/>
-    <tableColumn id="17" xr3:uid="{3D30E15F-1B0A-4446-9BD7-F4008384352E}" name="best iteration model file path" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{3318AD16-53B6-4688-8184-DCAE4D7989CC}" name="test number" dataDxfId="30"/>
+    <tableColumn id="26" xr3:uid="{36FCCC2D-6AA9-4D59-9607-CFE4E77F428F}" name="model iteration" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{6162A6E9-56C2-4DFE-8497-138E33277B23}" name="folders" dataDxfId="28"/>
+    <tableColumn id="24" xr3:uid="{84500DC1-61E5-441B-9BB7-98403DAEDDA3}" name="single or multi label" dataDxfId="27"/>
+    <tableColumn id="23" xr3:uid="{D53465F0-58BB-492A-A264-D9F6F9AD3C77}" name="file rating threshold" dataDxfId="26"/>
+    <tableColumn id="28" xr3:uid="{8B631FC7-380A-498A-87D1-A5A5CDE1B184}" name="sampling rate (hz)" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{455DD90A-7B3B-4AE3-B08F-EF626809FA12}" name="sound length (secs)" dataDxfId="24"/>
+    <tableColumn id="16" xr3:uid="{BE562B7A-09E8-48B6-87F1-F9358A9B6D5B}" name="files per folder threshold" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{E3C34C6B-84EB-4093-B2F3-6A3FEA8E014C}" name="sound clips per file threshold" dataDxfId="22"/>
+    <tableColumn id="27" xr3:uid="{191D39FF-C4F8-4DBA-B0D0-9163B957A029}" name="variance threshold" dataDxfId="21"/>
+    <tableColumn id="25" xr3:uid="{E5B8107D-0DF4-4EA1-ADD9-375779D45EF4}" name="mean db threshold" dataDxfId="20"/>
+    <tableColumn id="19" xr3:uid="{864FBBD1-F7F9-4946-B210-D69AFB5835DC}" name="test size" dataDxfId="19"/>
+    <tableColumn id="22" xr3:uid="{2B2C8707-3EBF-4F34-8873-79CDF32B12F6}" name="sampling" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{F22E151A-20C9-4BD4-9330-289A7FFEA185}" name="sound clips" dataDxfId="17"/>
+    <tableColumn id="18" xr3:uid="{5798ECBB-EF37-49E5-8484-9B35165F789E}" name="epochs" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{FCBAD803-5AC6-4170-96E5-CDADD42AAFE6}" name="loss function" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{28105F38-9933-41DD-903D-59C6CB55BAC1}" name="optimizer" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{EB347492-3ECD-4D09-9D3B-70F1B3841DE0}" name="learning rate" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{E8435981-3E1D-4BD4-B5A5-B92A95E47B32}" name="momentum" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{6CFBA716-45FB-401C-A304-C38379448F6E}" name="dropout rate" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{696423D6-C6E9-46A6-845B-0AF07B48592B}" name="batch size" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{7FD1D4E4-3292-4AA1-9BCC-2B94A81E0391}" name="training accuracy %" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{8EE7A374-9D10-4C25-9169-E97C46453BAF}" name="testing accuracy %" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{E1A45F5D-7C07-400E-8A62-BFF33A480A4C}" name="gpu train time (secs)" dataDxfId="7"/>
+    <tableColumn id="20" xr3:uid="{B80BC466-5D5A-48F1-9455-63991D7EF174}" name="top-5 accuracy" dataDxfId="6"/>
+    <tableColumn id="21" xr3:uid="{E7EF58AA-8977-49AA-AE41-D484359C41A5}" name="tested on?" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{26BF47AC-1BE1-47B7-86FA-94CD5B2EA529}" name="other changes" dataDxfId="4"/>
+    <tableColumn id="17" xr3:uid="{3D30E15F-1B0A-4446-9BD7-F4008384352E}" name="best iteration model file path" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1400,10 +1331,10 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="21.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="25.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="29.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -11459,8 +11390,8 @@
       <c r="X120" s="2">
         <v>746</v>
       </c>
-      <c r="Y120" s="2" t="s">
-        <v>146</v>
+      <c r="Y120" s="7">
+        <v>0.62180000000000002</v>
       </c>
       <c r="Z120" s="11" t="s">
         <v>65</v>
@@ -11714,7 +11645,7 @@
         <v>65</v>
       </c>
       <c r="AA123" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AB123" s="2"/>
     </row>
@@ -12208,7 +12139,7 @@
         <v>65</v>
       </c>
       <c r="AA129" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AB129" s="2"/>
     </row>
@@ -13030,7 +12961,7 @@
         <v>65</v>
       </c>
       <c r="AA139" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AB139" s="2"/>
     </row>
@@ -13196,7 +13127,7 @@
         <v>65</v>
       </c>
       <c r="AA141" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AB141" s="2"/>
     </row>
@@ -13222,7 +13153,7 @@
       <c r="G142" s="1">
         <v>2</v>
       </c>
-      <c r="H142" s="16">
+      <c r="H142" s="1">
         <v>20</v>
       </c>
       <c r="I142" s="1">
@@ -13280,7 +13211,7 @@
         <v>65</v>
       </c>
       <c r="AA142" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AB142" s="2"/>
     </row>
@@ -13304,8 +13235,9 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>